<commit_message>
style: make social signals platform filters dynamic and update local post insights
</commit_message>
<xml_diff>
--- a/News_Dashboard/data/social_media_posts.xlsx
+++ b/News_Dashboard/data/social_media_posts.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,77 +417,77 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Base_Company</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Competitor</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Author/Handle</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Date Created</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Post Text</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Image URL</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Image Text</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Video URL</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Video Transcript</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Post URL</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Sentiment</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Alert Level</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>AI Summary</t>
         </is>
@@ -7316,10 +7304,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>[Transcript unavailable: 
-Could not retrieve a transcript for the video https://www.youtube.com/watch?v=M6MP4urwaBw! This is most likely caused by:
-Subtitles are disabled for this video
-If you are sure that the described cause is not responsible for this error and that a transcript should be retrievable, please create an issue at https://github.com/jdepoix/youtube-transcript-api/issues. Please add which version of youtube_transcript_api you are using and provide the information needed to replicate the error. Also make sure that there are no open issues which already describe your problem!]</t>
+          <t>[Failed to fetch]</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -9228,17 +9213,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>[Transcript unavailable: 
-Could not retrieve a transcript for the video https://www.youtube.com/watch?v=FqYh9C_W-I4! This is most likely caused by:
-No transcripts were found for any of the requested language codes: ('en',)
-For this video (FqYh9C_W-I4) transcripts are available in the following languages:
-(MANUALLY CREATED)
-None
-(GENERATED)
- - vi ("Vietnamese (auto-generated)")[TRANSLATABLE]
-(TRANSLATION LANGUAGES)
- - en ("English")
-If you are sure that the described cause is not responsible for this error and that a transcript should be retrievable, please create an issue at https://github.com/jdepoix/youtube-transcript-api/issues. Please add which version of youtube_transcript_api you are using and provide the information needed to replicate the error. Also make sure that there are no open issues which already describe your problem!]</t>
+          <t>[Failed to fetch]</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -9292,7 +9267,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>[music] &gt;&gt; Oh. Hey, what's up?</t>
+          <t>[Failed to fetch]</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -27066,22 +27041,22 @@
       </c>
       <c r="L424" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M424" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N424" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O424" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp teases an upcoming initiative or partnership with the Tokenmaxx community, indicating a new product or service rollout.</t>
         </is>
       </c>
     </row>
@@ -27128,12 +27103,12 @@
       </c>
       <c r="L425" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M425" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N425" t="inlineStr">
@@ -27143,7 +27118,7 @@
       </c>
       <c r="O425" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp is offering a free service or promotion to user @karimatiyeh, indicating a partnership or promotional initiative.</t>
         </is>
       </c>
     </row>
@@ -27189,22 +27164,22 @@
       </c>
       <c r="L426" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M426" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N426" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O426" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp highlights a collaboration with @restocc and @eglyman, suggesting a potential partnership or joint initiative.</t>
         </is>
       </c>
     </row>
@@ -27250,12 +27225,12 @@
       </c>
       <c r="L427" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M427" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N427" t="inlineStr">
@@ -27265,7 +27240,7 @@
       </c>
       <c r="O427" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp mentions @pontusab, likely indicating a partnership or collaboration announcement.</t>
         </is>
       </c>
     </row>
@@ -27313,22 +27288,22 @@
       </c>
       <c r="L428" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M428" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Tech Updates</t>
         </is>
       </c>
       <c r="N428" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O428" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp announced a data‑driven analysis of spending profiles, detailing variations in model choices, caching habits, prompts, and spend controls, and invites users to compare their own usage.</t>
         </is>
       </c>
     </row>
@@ -27376,22 +27351,22 @@
       </c>
       <c r="L429" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M429" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N429" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O429" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp promotes a new AI spend management feature that connects business data, tracks team trends, and maximizes token value.</t>
         </is>
       </c>
     </row>
@@ -27437,12 +27412,12 @@
       </c>
       <c r="L430" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M430" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Leadership Changes</t>
         </is>
       </c>
       <c r="N430" t="inlineStr">
@@ -27452,7 +27427,7 @@
       </c>
       <c r="O430" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp shares a playful tweet acknowledging its CFO, expressing appreciation.</t>
         </is>
       </c>
     </row>
@@ -27513,7 +27488,7 @@
       </c>
       <c r="O431" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex data reveals that three of the top 25 most-purchased founder books this year are from Stripe Press, with two more just outside the list, underscoring the press's growing influence among startup founders.</t>
         </is>
       </c>
     </row>
@@ -27574,7 +27549,7 @@
       </c>
       <c r="O432" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex reports shifts in the popularity of books among its founders, with Atomic Habits falling in rank while titles like High Output Management and The Hard Thing About Hard Things rise.</t>
         </is>
       </c>
     </row>
@@ -27635,7 +27610,7 @@
       </c>
       <c r="O433" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex shares data revealing that founders’ purchasing habits reflect their interests, with the most popular business book among Brex cardholders in H1 2026 being a new biography of Alex Karp.</t>
         </is>
       </c>
     </row>
@@ -27681,12 +27656,12 @@
       </c>
       <c r="L434" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M434" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N434" t="inlineStr">
@@ -27696,7 +27671,7 @@
       </c>
       <c r="O434" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex teases a collaboration with several wine industry influencers, indicating a new partnership or initiative.</t>
         </is>
       </c>
     </row>
@@ -27782,7 +27757,7 @@
       </c>
       <c r="O435" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex posted a curated list of business and leadership books, showcasing resources for professional development and thought leadership.</t>
         </is>
       </c>
     </row>
@@ -27845,7 +27820,7 @@
       </c>
       <c r="O436" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex reports that founder biographies are the top book choice among its 35,000+ customers, with a shift toward AI in management frameworks noted in H1 2026 rankings.</t>
         </is>
       </c>
     </row>
@@ -27901,12 +27876,12 @@
       </c>
       <c r="L437" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M437" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N437" t="inlineStr">
@@ -27916,7 +27891,7 @@
       </c>
       <c r="O437" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Airbnb partnered with Heartshare and supported 50 foster youth to attend a 2026 FIFA World Cup match, showcasing its commitment to community engagement and youth empowerment.</t>
         </is>
       </c>
     </row>
@@ -27966,12 +27941,12 @@
       </c>
       <c r="L438" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M438" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N438" t="inlineStr">
@@ -27981,7 +27956,7 @@
       </c>
       <c r="O438" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Expedia promotes a Norwegian travel package featuring fjords, midnight sun hikes, and cabin stays, encouraging bookings through a provided link.</t>
         </is>
       </c>
     </row>
@@ -28043,12 +28018,12 @@
       </c>
       <c r="L439" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M439" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N439" t="inlineStr">
@@ -28058,7 +28033,7 @@
       </c>
       <c r="O439" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Expedia promotes a curated Big Sur road‑trip itinerary and highlights booking perks such as OneKeyCash and future travel benefits to entice users to book through its platform.</t>
         </is>
       </c>
     </row>
@@ -28119,7 +28094,7 @@
       </c>
       <c r="O440" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs users that flight reservations cannot be handled via social media and directs them to contact the Flights team via a provided link or phone numbers.</t>
         </is>
       </c>
     </row>
@@ -28165,7 +28140,7 @@
       </c>
       <c r="L441" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M441" t="inlineStr">
@@ -28180,7 +28155,7 @@
       </c>
       <c r="O441" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user complaint about flight reservation assistance, citing GDPR and security restrictions that prevent them from providing help on social media and advising the user to contact the flight team again.</t>
         </is>
       </c>
     </row>
@@ -28227,7 +28202,7 @@
       </c>
       <c r="L442" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M442" t="inlineStr">
@@ -28242,7 +28217,7 @@
       </c>
       <c r="O442" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user’s inquiry, offering help and directing them to a specialized support team.</t>
         </is>
       </c>
     </row>
@@ -28317,7 +28292,7 @@
       </c>
       <c r="O443" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com reiterates its customer data protection policies, clarifying that it does not request credit card details via phone or email, does not use WhatsApp for support, and provides official communication channels.</t>
         </is>
       </c>
     </row>
@@ -28378,7 +28353,7 @@
       </c>
       <c r="O444" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s direct message, indicating routine customer support activity.</t>
         </is>
       </c>
     </row>
@@ -28439,7 +28414,7 @@
       </c>
       <c r="O445" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint about a pending refund, directing them to the Flights team for assistance.</t>
         </is>
       </c>
     </row>
@@ -28506,7 +28481,7 @@
       </c>
       <c r="O446" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is following up with a customer about a car rental reservation, requesting booking details for assistance.</t>
         </is>
       </c>
     </row>
@@ -28573,7 +28548,7 @@
       </c>
       <c r="O447" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com sent a follow‑up message to a customer about a car rental reservation, requesting booking details to provide assistance.</t>
         </is>
       </c>
     </row>
@@ -28641,7 +28616,7 @@
       </c>
       <c r="O448" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com explains its social media support process for accommodation bookings, offering private messaging and phone contact, and directs other inquiries to specialized teams.</t>
         </is>
       </c>
     </row>
@@ -28703,7 +28678,7 @@
       </c>
       <c r="O449" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replies to a user’s request for assistance with a standard policy statement, directing them to the collaborator help center.</t>
         </is>
       </c>
     </row>
@@ -28767,7 +28742,7 @@
       </c>
       <c r="O450" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is offering customer support instructions for a user regarding reservation confirmation details and providing a phone contact link.</t>
         </is>
       </c>
     </row>
@@ -28813,7 +28788,7 @@
       </c>
       <c r="L451" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M451" t="inlineStr">
@@ -28828,7 +28803,7 @@
       </c>
       <c r="O451" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replies to a dissatisfied user on X, expressing regret and offering to assist via private message.</t>
         </is>
       </c>
     </row>
@@ -28889,7 +28864,7 @@
       </c>
       <c r="O452" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a delayed response to a user, citing a high volume of social media inquiries.</t>
         </is>
       </c>
     </row>
@@ -28950,7 +28925,7 @@
       </c>
       <c r="O453" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user about a flight delay, offering alternative contact methods for assistance.</t>
         </is>
       </c>
     </row>
@@ -29015,7 +28990,7 @@
       </c>
       <c r="O454" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com addresses a customer complaint about a property, offering support and clarifying its intermediary role.</t>
         </is>
       </c>
     </row>
@@ -29076,7 +29051,7 @@
       </c>
       <c r="O455" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com sent a private message to user @tdog1410, requesting them to check their private message.</t>
         </is>
       </c>
     </row>
@@ -29128,7 +29103,7 @@
       </c>
       <c r="M456" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Tech Updates</t>
         </is>
       </c>
       <c r="N456" t="inlineStr">
@@ -29138,7 +29113,7 @@
       </c>
       <c r="O456" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user complaint about potentially false property listings, outlining its verification process and offering to investigate and remove inaccurate listings.</t>
         </is>
       </c>
     </row>
@@ -29204,7 +29179,7 @@
       </c>
       <c r="O457" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user’s refund concern via X, offering details to resolve the issue and directing to 24/7 customer service for immediate support.</t>
         </is>
       </c>
     </row>
@@ -29269,7 +29244,7 @@
       </c>
       <c r="O458" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replies to a customer complaint, clarifying that it acts as an intermediary and offering to assist with further details.</t>
         </is>
       </c>
     </row>
@@ -29333,7 +29308,7 @@
       </c>
       <c r="O459" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint about a non‑refundable cancellation in Prague, explaining that cancellation policies are managed by property owners and offering to contact the property on the customer’s behalf.</t>
         </is>
       </c>
     </row>
@@ -29395,12 +29370,12 @@
       </c>
       <c r="L460" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M460" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N460" t="inlineStr">
@@ -29410,7 +29385,7 @@
       </c>
       <c r="O460" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com promotes a new pet-friendly vacation concept, emphasizing a hassle‑free, drama‑free experience for travelers with cats.</t>
         </is>
       </c>
     </row>
@@ -29468,7 +29443,7 @@
       </c>
       <c r="L461" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M461" t="inlineStr">
@@ -29483,7 +29458,7 @@
       </c>
       <c r="O461" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Expedia promotes Croatia as a top summer destination, offering travel tips for Plitvice Lakes, island hopping, and highlighting the new Euro currency.</t>
         </is>
       </c>
     </row>
@@ -29548,7 +29523,7 @@
       </c>
       <c r="O462" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a property’s failure to accommodate a guest and offers assistance in finding alternative accommodation, providing contact details for support.</t>
         </is>
       </c>
     </row>
@@ -29609,7 +29584,7 @@
       </c>
       <c r="O463" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s concern via direct message, indicating they have addressed the issue.</t>
         </is>
       </c>
     </row>
@@ -29661,7 +29636,7 @@
       </c>
       <c r="M464" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Tech Updates</t>
         </is>
       </c>
       <c r="N464" t="inlineStr">
@@ -29671,7 +29646,7 @@
       </c>
       <c r="O464" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com acknowledges a limitation in its platform’s filtering options, apologizing for not being able to filter by check‑in or check‑out times and expressing appreciation for user feedback.</t>
         </is>
       </c>
     </row>
@@ -29733,7 +29708,7 @@
       </c>
       <c r="O465" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replies to a user on X, apologizing for a delayed response and directing them to a private message.</t>
         </is>
       </c>
     </row>
@@ -29780,7 +29755,7 @@
       </c>
       <c r="L466" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M466" t="inlineStr">
@@ -29795,7 +29770,7 @@
       </c>
       <c r="O466" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes to user Roberto for an issue and expresses hope for a quick resolution.</t>
         </is>
       </c>
     </row>
@@ -29842,7 +29817,7 @@
       </c>
       <c r="L467" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M467" t="inlineStr">
@@ -29857,7 +29832,7 @@
       </c>
       <c r="O467" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com thanks a user for their feedback and offers future assistance, highlighting its customer service approach.</t>
         </is>
       </c>
     </row>
@@ -29903,12 +29878,12 @@
       </c>
       <c r="L468" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M468" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N468" t="inlineStr">
@@ -29918,7 +29893,7 @@
       </c>
       <c r="O468" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex is promoting a watch party event, likely to showcase a new product or feature to its audience.</t>
         </is>
       </c>
     </row>
@@ -29965,7 +29940,7 @@
       </c>
       <c r="L469" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M469" t="inlineStr">
@@ -29980,7 +29955,7 @@
       </c>
       <c r="O469" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex is promoting a watch party for the Finance On Offense Finals, targeting audiences in Spain and Argentina.</t>
         </is>
       </c>
     </row>
@@ -30034,7 +30009,7 @@
       </c>
       <c r="L470" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M470" t="inlineStr">
@@ -30049,7 +30024,7 @@
       </c>
       <c r="O470" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Airbnb celebrates Spain’s World Cup victory and promotes travel to Spain with a celebratory post.</t>
         </is>
       </c>
     </row>
@@ -30110,7 +30085,7 @@
       </c>
       <c r="O471" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs partners that it cannot provide support via social media and directs them to its Partner Support contact page.</t>
         </is>
       </c>
     </row>
@@ -30176,7 +30151,7 @@
       </c>
       <c r="O472" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user’s inquiry about flight reservations, apologizing for the inconvenience and directing them to the Flights team via a link and phone numbers.</t>
         </is>
       </c>
     </row>
@@ -30237,7 +30212,7 @@
       </c>
       <c r="O473" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a refund inquiry, directing the customer to the dedicated Flights team and providing contact details, citing GDPR restrictions.</t>
         </is>
       </c>
     </row>
@@ -30286,7 +30261,7 @@
       </c>
       <c r="L474" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M474" t="inlineStr">
@@ -30301,7 +30276,7 @@
       </c>
       <c r="O474" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replies to a user on X, stating it cannot help via social media and directs the inquiry to a specialized team.</t>
         </is>
       </c>
     </row>
@@ -30362,7 +30337,7 @@
       </c>
       <c r="O475" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user’s complaint about a reservation issue, offering to resolve it via another profile to avoid confusion.</t>
         </is>
       </c>
     </row>
@@ -30424,7 +30399,7 @@
       </c>
       <c r="O476" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s private message, apologizing for an issue.</t>
         </is>
       </c>
     </row>
@@ -30488,7 +30463,7 @@
       </c>
       <c r="O477" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint, offering to connect with customer service and providing instructions for escalation.</t>
         </is>
       </c>
     </row>
@@ -30551,7 +30526,7 @@
       </c>
       <c r="O478" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is responding to a user’s request for reservation details, asking for the pin code via private message.</t>
         </is>
       </c>
     </row>
@@ -30616,7 +30591,7 @@
       </c>
       <c r="O479" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is responding to a user’s complaint about missing check‑in details, requesting confirmation number, email, and guest name via private message.</t>
         </is>
       </c>
     </row>
@@ -30677,7 +30652,7 @@
       </c>
       <c r="O480" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs a user that they have sent a private message, indicating a direct outreach or marketing effort.</t>
         </is>
       </c>
     </row>
@@ -30738,7 +30713,7 @@
       </c>
       <c r="O481" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied privately to a user, directing them to check their direct messages.</t>
         </is>
       </c>
     </row>
@@ -30799,7 +30774,7 @@
       </c>
       <c r="O482" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs a user that accommodation bookings can be handled via social media, but flight requests must be directed to a dedicated flight support team.</t>
         </is>
       </c>
     </row>
@@ -30860,7 +30835,7 @@
       </c>
       <c r="O483" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s direct message, indicating ongoing customer engagement.</t>
         </is>
       </c>
     </row>
@@ -30921,7 +30896,7 @@
       </c>
       <c r="O484" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com provides a user with instructions on how to find contact numbers and call customer support.</t>
         </is>
       </c>
     </row>
@@ -30982,7 +30957,7 @@
       </c>
       <c r="O485" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com posted a brief tweet indicating it has sent a direct message to a user named David.</t>
         </is>
       </c>
     </row>
@@ -31033,7 +31008,7 @@
       </c>
       <c r="M486" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N486" t="inlineStr">
@@ -31043,7 +31018,7 @@
       </c>
       <c r="O486" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs partners that it cannot provide support via social media and directs them to its Partner Support contact page.</t>
         </is>
       </c>
     </row>
@@ -31089,7 +31064,7 @@
       </c>
       <c r="L487" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M487" t="inlineStr">
@@ -31104,7 +31079,7 @@
       </c>
       <c r="O487" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user with a courteous thank‑you and well‑wishes.</t>
         </is>
       </c>
     </row>
@@ -31165,7 +31140,7 @@
       </c>
       <c r="O488" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs customers that flight changes cannot be handled via X and directs them to the Flights team for assistance.</t>
         </is>
       </c>
     </row>
@@ -31212,7 +31187,7 @@
       </c>
       <c r="L489" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M489" t="inlineStr">
@@ -31227,7 +31202,7 @@
       </c>
       <c r="O489" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com explains that check‑in and check‑out times are set by each property and advises customers to review details and contact the property for early check‑in or late check‑out options.</t>
         </is>
       </c>
     </row>
@@ -31273,7 +31248,7 @@
       </c>
       <c r="L490" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M490" t="inlineStr">
@@ -31288,7 +31263,7 @@
       </c>
       <c r="O490" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user offering immediate assistance via a phone link.</t>
         </is>
       </c>
     </row>
@@ -31334,12 +31309,12 @@
       </c>
       <c r="L491" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M491" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N491" t="inlineStr">
@@ -31349,7 +31324,7 @@
       </c>
       <c r="O491" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Navan promotes a case study that showcases the effectiveness of its product.</t>
         </is>
       </c>
     </row>
@@ -31397,22 +31372,22 @@
       </c>
       <c r="L492" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M492" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N492" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O492" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Navan highlights its partnership with Adyen, showcasing its ability to streamline large-scale corporate travel logistics and reduce manual coordination for a global workforce.</t>
         </is>
       </c>
     </row>
@@ -31458,22 +31433,22 @@
       </c>
       <c r="L493" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M493" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N493" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O493" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp highlights a 3D animated video showcasing their new construction product launch, emphasizing creative marketing and product visibility.</t>
         </is>
       </c>
     </row>
@@ -31534,7 +31509,7 @@
       </c>
       <c r="O494" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp posted a tweet referencing an art piece by @iamjasonlevin.</t>
         </is>
       </c>
     </row>
@@ -31595,7 +31570,7 @@
       </c>
       <c r="O495" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex’s tweet mentions @tobiwaldhecker, likely indicating a brief acknowledgment or potential collaboration, but no specific announcement is evident.</t>
         </is>
       </c>
     </row>
@@ -31641,12 +31616,12 @@
       </c>
       <c r="L496" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M496" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N496" t="inlineStr">
@@ -31656,7 +31631,7 @@
       </c>
       <c r="O496" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex emphasizes the drawbacks of manual expense reports, positioning its solution as a more efficient alternative.</t>
         </is>
       </c>
     </row>
@@ -31717,7 +31692,7 @@
       </c>
       <c r="O497" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex posts a brief, inquisitive remark to @anieasyy, indicating curiosity about a prior event or post.</t>
         </is>
       </c>
     </row>
@@ -31778,7 +31753,7 @@
       </c>
       <c r="O498" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex posted a generic greeting 'top of the morning' with no substantive content.</t>
         </is>
       </c>
     </row>
@@ -31824,12 +31799,12 @@
       </c>
       <c r="L499" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M499" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N499" t="inlineStr">
@@ -31839,7 +31814,7 @@
       </c>
       <c r="O499" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex publicly thanks PigPugHealth for joining them, signaling a new partnership or collaboration.</t>
         </is>
       </c>
     </row>
@@ -31885,7 +31860,7 @@
       </c>
       <c r="L500" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M500" t="inlineStr">
@@ -31900,7 +31875,7 @@
       </c>
       <c r="O500" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Airbnb celebrates a fulfilled promise with chef Jose Andres, referencing a World Cup victory.</t>
         </is>
       </c>
     </row>
@@ -31962,7 +31937,7 @@
       </c>
       <c r="L501" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M501" t="inlineStr">
@@ -31977,7 +31952,7 @@
       </c>
       <c r="O501" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Airbnb highlights global unity and community spirit during the World Cup, encouraging continued engagement and hinting at future events in Brazil 2027.</t>
         </is>
       </c>
     </row>
@@ -32038,7 +32013,7 @@
       </c>
       <c r="O502" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com sent a private message to user @Mandy60029581, prompting them to check their inbox.</t>
         </is>
       </c>
     </row>
@@ -32100,7 +32075,7 @@
       </c>
       <c r="O503" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is responding to a customer complaint, offering to investigate the issue via private message.</t>
         </is>
       </c>
     </row>
@@ -32165,7 +32140,7 @@
       </c>
       <c r="O504" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer inquiry on X, requesting reservation details and directing the user to 24/7 support for immediate assistance.</t>
         </is>
       </c>
     </row>
@@ -32226,7 +32201,7 @@
       </c>
       <c r="O505" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint about payment options, clarifying that partners accept various payment methods and directing the user to a private message for further details.</t>
         </is>
       </c>
     </row>
@@ -32293,7 +32268,7 @@
       </c>
       <c r="O506" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is offering refund assistance to a customer via private message.</t>
         </is>
       </c>
     </row>
@@ -32357,7 +32332,7 @@
       </c>
       <c r="O507" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is responding to a customer complaint about a pending refund, requesting account details via DM to investigate the issue.</t>
         </is>
       </c>
     </row>
@@ -32418,7 +32393,7 @@
       </c>
       <c r="O508" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s DM, offering further assistance.</t>
         </is>
       </c>
     </row>
@@ -32484,7 +32459,7 @@
       </c>
       <c r="O509" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint, apologizing and requesting private details for further investigation.</t>
         </is>
       </c>
     </row>
@@ -32531,22 +32506,22 @@
       </c>
       <c r="L510" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M510" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N510" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O510" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Sky Bird Travel promotes a new nonstop Los Angeles–Casablanca flight via Royal Air Maroc, aiming to increase sales across Morocco, Africa, Europe, and Asia.</t>
         </is>
       </c>
     </row>
@@ -32602,12 +32577,12 @@
       </c>
       <c r="L511" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M511" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N511" t="inlineStr">
@@ -32617,7 +32592,7 @@
       </c>
       <c r="O511" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Sky Bird Travel is promoting a new nonstop Los Angeles–Casablanca service with Royal Air Maroc, urging travel agents to book via WINGS.</t>
         </is>
       </c>
     </row>
@@ -32681,22 +32656,22 @@
       </c>
       <c r="L512" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M512" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Strategic Expansion or Changes</t>
         </is>
       </c>
       <c r="N512" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O512" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Navan announces the opening of a new office overseas, emphasizing its role in simplifying coordination for a senior manager at Adyen. The post showcases how the platform enables focus on key moments during global expansion.</t>
         </is>
       </c>
     </row>
@@ -32744,12 +32719,12 @@
       </c>
       <c r="L513" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M513" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N513" t="inlineStr">
@@ -32759,7 +32734,7 @@
       </c>
       <c r="O513" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp announces that more than 1,000 businesses use its stablecoin payment service, with over 70% of the volume moving outside traditional banking hours, and invites new users to open a stablecoin account.</t>
         </is>
       </c>
     </row>
@@ -32809,22 +32784,22 @@
       </c>
       <c r="L514" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M514" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N514" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O514" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp announces the addition of stablecoins (USDC and USDT) to its platform, enabling faster cross-border vendor payments with existing approval and accounting workflows.</t>
         </is>
       </c>
     </row>
@@ -32885,7 +32860,7 @@
       </c>
       <c r="O515" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp posted a nonsensical tweet with repeated words, providing no meaningful information.</t>
         </is>
       </c>
     </row>
@@ -32931,12 +32906,12 @@
       </c>
       <c r="L516" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M516" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Leadership Changes</t>
         </is>
       </c>
       <c r="N516" t="inlineStr">
@@ -32946,7 +32921,7 @@
       </c>
       <c r="O516" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp publicly acknowledges @sridvijay’s new role or partnership, expressing gratitude and honor.</t>
         </is>
       </c>
     </row>
@@ -32993,22 +32968,22 @@
       </c>
       <c r="L517" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M517" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Tech Updates</t>
         </is>
       </c>
       <c r="N517" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O517" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp claims to have reduced its AI expenses by 30% with a router that selects the optimal model for each task, positioning the solution as a cost‑saving option for others.</t>
         </is>
       </c>
     </row>
@@ -33054,7 +33029,7 @@
       </c>
       <c r="L518" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M518" t="inlineStr">
@@ -33069,7 +33044,7 @@
       </c>
       <c r="O518" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp shares a supportive message towards @rahulgs, indicating positive engagement.</t>
         </is>
       </c>
     </row>
@@ -33115,12 +33090,12 @@
       </c>
       <c r="L519" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M519" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N519" t="inlineStr">
@@ -33130,7 +33105,7 @@
       </c>
       <c r="O519" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex promotes its collaboration with @vibedotco, highlighting how the partnership helped achieve a specific goal.</t>
         </is>
       </c>
     </row>
@@ -33177,22 +33152,22 @@
       </c>
       <c r="L520" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M520" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N520" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O520" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex used its points program to fund a $128,000 out‑of‑home advertising campaign in partnership with vibedotco, creating a viral campaign without additional spend.</t>
         </is>
       </c>
     </row>
@@ -33238,7 +33213,7 @@
       </c>
       <c r="L521" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M521" t="inlineStr">
@@ -33253,7 +33228,7 @@
       </c>
       <c r="O521" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex highlights @zachmoskow with a fire emoji, signaling enthusiasm or support.</t>
         </is>
       </c>
     </row>
@@ -33299,12 +33274,12 @@
       </c>
       <c r="L522" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M522" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N522" t="inlineStr">
@@ -33314,7 +33289,7 @@
       </c>
       <c r="O522" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex publicly thanks Fondocom for a shout, indicating a positive partnership or collaboration.</t>
         </is>
       </c>
     </row>
@@ -33365,7 +33340,7 @@
       </c>
       <c r="M523" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N523" t="inlineStr">
@@ -33375,7 +33350,7 @@
       </c>
       <c r="O523" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex acknowledges a collaboration with Telnyx, suggesting a partnership aimed at maintaining operational stability.</t>
         </is>
       </c>
     </row>
@@ -33431,12 +33406,12 @@
       </c>
       <c r="L524" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M524" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N524" t="inlineStr">
@@ -33446,7 +33421,7 @@
       </c>
       <c r="O524" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>AirBnb celebrates global unity at the 2026 FIFA World Cup and hints at continuing engagement in Brazil in 2027.</t>
         </is>
       </c>
     </row>
@@ -33500,12 +33475,12 @@
       </c>
       <c r="L525" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M525" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N525" t="inlineStr">
@@ -33515,7 +33490,7 @@
       </c>
       <c r="O525" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Expedia showcases its Island Hot List, promoting new summer getaways and inviting followers to pick their next destination.</t>
         </is>
       </c>
     </row>
@@ -33572,22 +33547,22 @@
       </c>
       <c r="L526" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M526" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N526" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O526" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Expedia unveils its 2026 Island Hot List of 10 emerging island destinations and runs a £3,500 prize contest for a Cosmo Club member to win an island getaway.</t>
         </is>
       </c>
     </row>
@@ -33636,12 +33611,12 @@
       </c>
       <c r="L527" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M527" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N527" t="inlineStr">
@@ -33651,7 +33626,7 @@
       </c>
       <c r="O527" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Expedia unveiled its 2026 Island Hot List, highlighting ten emerging island destinations and promoting bundled flight+hotel deals to attract travelers.</t>
         </is>
       </c>
     </row>
@@ -33715,7 +33690,7 @@
       </c>
       <c r="O528" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is responding to a customer complaint, requesting private details to investigate the issue.</t>
         </is>
       </c>
     </row>
@@ -33776,12 +33751,12 @@
       </c>
       <c r="N529" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O529" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com cautions guests not to share personal details on unrecognized channels and offers to investigate potential security incidents.</t>
         </is>
       </c>
     </row>
@@ -33845,7 +33820,7 @@
       </c>
       <c r="O530" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replies to a user’s complaint, asking for private details to resolve the issue.</t>
         </is>
       </c>
     </row>
@@ -33908,7 +33883,7 @@
       </c>
       <c r="O531" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint about a pending refund, directing them to the flight booking support channel.</t>
         </is>
       </c>
     </row>
@@ -33970,12 +33945,12 @@
       </c>
       <c r="N532" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O532" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a delayed response to a user’s complaint about a double charge and requests booking details via private message.</t>
         </is>
       </c>
     </row>
@@ -34036,7 +34011,7 @@
       </c>
       <c r="O533" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a private message from user @iklswsk regarding an unspecified issue.</t>
         </is>
       </c>
     </row>
@@ -34102,7 +34077,7 @@
       </c>
       <c r="O534" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is outlining its customer support process, encouraging users to send private messages with reservation details and directing them to 24/7 support for immediate assistance.</t>
         </is>
       </c>
     </row>
@@ -34168,7 +34143,7 @@
       </c>
       <c r="O535" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint on X, offering private message support and directing users to 24/7 phone support, while clarifying that only accommodation bookings are handled via social media.</t>
         </is>
       </c>
     </row>
@@ -34230,7 +34205,7 @@
       </c>
       <c r="O536" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs users that flight bookings cannot be handled via X and directs them to contact the flight team via link or phone.</t>
         </is>
       </c>
     </row>
@@ -34296,7 +34271,7 @@
       </c>
       <c r="O537" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com addresses a customer’s difficulty reaching its customer care team, offering a direct message format for booking inquiries and providing a local phone number.</t>
         </is>
       </c>
     </row>
@@ -34346,7 +34321,7 @@
       </c>
       <c r="L538" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M538" t="inlineStr">
@@ -34361,7 +34336,7 @@
       </c>
       <c r="O538" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com addresses a customer complaint about being charged twice, offering to investigate via direct message and directing the user to 24/7 customer support.</t>
         </is>
       </c>
     </row>
@@ -34426,7 +34401,7 @@
       </c>
       <c r="O539" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is responding to a customer inquiry about reviewing a booking, providing instructions for the customer to send details via DM.</t>
         </is>
       </c>
     </row>
@@ -34493,7 +34468,7 @@
       </c>
       <c r="O540" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user complaint, offering to resolve issues via private message or phone.</t>
         </is>
       </c>
     </row>
@@ -34557,7 +34532,7 @@
       </c>
       <c r="O541" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com addresses a user’s pending refund request, asking for confirmation details via private message.</t>
         </is>
       </c>
     </row>
@@ -34607,22 +34582,22 @@
       </c>
       <c r="L542" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M542" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Tech Updates</t>
         </is>
       </c>
       <c r="N542" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O542" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com highlights its ongoing security measures, including 24/7 monitoring and compliance checks, to reassure clients and partners about the safety of listings on its platform.</t>
         </is>
       </c>
     </row>
@@ -34689,7 +34664,7 @@
       </c>
       <c r="O543" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com addresses a customer complaint on X, offering to review the booking and directing the user to further support channels.</t>
         </is>
       </c>
     </row>
@@ -34751,7 +34726,7 @@
       </c>
       <c r="O544" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com publicly apologized to a user for an issue with a reservation and noted that they responded via private message.</t>
         </is>
       </c>
     </row>
@@ -34798,7 +34773,7 @@
       </c>
       <c r="L545" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M545" t="inlineStr">
@@ -34813,7 +34788,7 @@
       </c>
       <c r="O545" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com declines to address a customer’s issue via social media, directing them to other support channels.</t>
         </is>
       </c>
     </row>
@@ -34877,7 +34852,7 @@
       </c>
       <c r="O546" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replies to a partner’s message, apologizing for the delay and directing them to secure support channels.</t>
         </is>
       </c>
     </row>
@@ -34939,7 +34914,7 @@
       </c>
       <c r="O547" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs partners that it cannot provide support via social media and directs them to a partner support contact page.</t>
         </is>
       </c>
     </row>
@@ -35000,7 +34975,7 @@
       </c>
       <c r="O548" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com for Travel Agents sent a private message to user @Ameerat_alwardd, requesting them to check it at their earliest convenience.</t>
         </is>
       </c>
     </row>
@@ -35049,7 +35024,7 @@
       </c>
       <c r="L549" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M549" t="inlineStr">
@@ -35064,7 +35039,7 @@
       </c>
       <c r="O549" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Navan announced it has been named one of the World’s Top Fintech Companies by CNBC and Statista, celebrating its growth and customer base.</t>
         </is>
       </c>
     </row>
@@ -35460,22 +35435,22 @@
       </c>
       <c r="L555" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M555" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N555" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O555" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp announces a partnership with Zebrie and Camille Ricketts, indicating a strategic collaboration.</t>
         </is>
       </c>
     </row>
@@ -35536,7 +35511,7 @@
       </c>
       <c r="O556" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp posted a brief, lighthearted comment referencing Figma’s design, with no clear business implication.</t>
         </is>
       </c>
     </row>
@@ -35582,7 +35557,7 @@
       </c>
       <c r="L557" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M557" t="inlineStr">
@@ -35597,7 +35572,7 @@
       </c>
       <c r="O557" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>A tweet claims that sources say Ramp is stable, suggesting a positive perception of the company's financial health.</t>
         </is>
       </c>
     </row>
@@ -35658,7 +35633,7 @@
       </c>
       <c r="O558" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp references a major key with @damianplayer, suggesting a potential partnership or collaboration.</t>
         </is>
       </c>
     </row>
@@ -35704,7 +35679,7 @@
       </c>
       <c r="L559" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M559" t="inlineStr">
@@ -35714,12 +35689,12 @@
       </c>
       <c r="N559" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O559" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp posted a sarcastic remark about Solana, claiming the post was fact‑checked by "real global stablecoin enjoyers," indicating a negative stance toward Solana.</t>
         </is>
       </c>
     </row>
@@ -35766,22 +35741,22 @@
       </c>
       <c r="L560" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M560" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N560" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O560" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex announces that AI agents can now receive their own corporate cards, highlighting a rapid rollout of this new feature.</t>
         </is>
       </c>
     </row>
@@ -35829,22 +35804,22 @@
       </c>
       <c r="L561" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M561" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N561" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O561" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex highlights a new self‑correcting agent pipeline built with @cursor_ai that dramatically speeds up manual framework upgrades, boosting efficiency by 32×.</t>
         </is>
       </c>
     </row>
@@ -35890,22 +35865,22 @@
       </c>
       <c r="L562" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M562" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N562" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O562" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex announces a new product or service aimed at expanding its corporate card and financial solutions.</t>
         </is>
       </c>
     </row>
@@ -35989,7 +35964,7 @@
       </c>
       <c r="O563" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex posted a brief Instagram update with emojis and unrelated car hashtags, indicating no significant activity or announcement.</t>
         </is>
       </c>
     </row>
@@ -36039,12 +36014,12 @@
       </c>
       <c r="L564" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M564" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N564" t="inlineStr">
@@ -36054,7 +36029,7 @@
       </c>
       <c r="O564" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Expedia promotes a travel package to Paraguay, highlighting historic ruins, cultural experiences, and unique colonial stays, and directs followers to book via a provided link.</t>
         </is>
       </c>
     </row>
@@ -36102,12 +36077,12 @@
       </c>
       <c r="L565" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M565" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N565" t="inlineStr">
@@ -36117,7 +36092,7 @@
       </c>
       <c r="O565" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Expedia is promoting a 10% discount on Disney Theme Park tickets with code DISNEY10, encouraging bookings before the offer expires.</t>
         </is>
       </c>
     </row>
@@ -36173,12 +36148,12 @@
       </c>
       <c r="L566" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M566" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N566" t="inlineStr">
@@ -36188,7 +36163,7 @@
       </c>
       <c r="O566" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Expedia promotes a set-jetting Greece trip featuring mythological sites and a traditional stone villa stay, encouraging followers to plan via a provided link.</t>
         </is>
       </c>
     </row>
@@ -36249,7 +36224,7 @@
       </c>
       <c r="O567" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com’s social media team informs a customer that they cannot see prior communications and requests booking details to proceed with assistance.</t>
         </is>
       </c>
     </row>
@@ -36311,7 +36286,7 @@
       </c>
       <c r="O568" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a private message from a user, acknowledging receipt and inviting them to review the response.</t>
         </is>
       </c>
     </row>
@@ -36372,7 +36347,7 @@
       </c>
       <c r="O569" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint, offering assistance via direct message.</t>
         </is>
       </c>
     </row>
@@ -36440,7 +36415,7 @@
       </c>
       <c r="O570" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a missing booking confirmation and requests customer details via DM to resolve the issue.</t>
         </is>
       </c>
     </row>
@@ -36506,7 +36481,7 @@
       </c>
       <c r="O571" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer inquiry about a pending refund, offering to review the booking and request additional details to expedite the process.</t>
         </is>
       </c>
     </row>
@@ -36572,7 +36547,7 @@
       </c>
       <c r="O572" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a hotel’s failure to accommodate a guest and offers assistance to resolve the issue.</t>
         </is>
       </c>
     </row>
@@ -36635,7 +36610,7 @@
       </c>
       <c r="O573" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com clarified that its social media channel only handles accommodation bookings and directed the user to a flight reservation contact link.</t>
         </is>
       </c>
     </row>
@@ -36701,7 +36676,7 @@
       </c>
       <c r="O574" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint, offering to gather booking details to resolve the issue.</t>
         </is>
       </c>
     </row>
@@ -36762,7 +36737,7 @@
       </c>
       <c r="O575" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs a user that flight reservations cannot be handled via social media and directs them to the Flights team contact details.</t>
         </is>
       </c>
     </row>
@@ -36829,7 +36804,7 @@
       </c>
       <c r="O576" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs customers that incomplete bookings may not have processed and offers steps to verify and correct booking details.</t>
         </is>
       </c>
     </row>
@@ -36894,7 +36869,7 @@
       </c>
       <c r="O577" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint, directing them to provide details via DM and encouraging direct communication with the property.</t>
         </is>
       </c>
     </row>
@@ -36940,7 +36915,7 @@
       </c>
       <c r="L578" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M578" t="inlineStr">
@@ -36955,7 +36930,7 @@
       </c>
       <c r="O578" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user, expressing satisfaction and offering further assistance.</t>
         </is>
       </c>
     </row>
@@ -37022,7 +36997,7 @@
       </c>
       <c r="O579" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a dissatisfied customer, offering to review the booking and requesting details via DM.</t>
         </is>
       </c>
     </row>
@@ -37088,7 +37063,7 @@
       </c>
       <c r="O580" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a refund inquiry on X, offering support for accommodation bookings and directing other service requests to dedicated teams.</t>
         </is>
       </c>
     </row>
@@ -37153,7 +37128,7 @@
       </c>
       <c r="O581" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint on X, offering to investigate and requesting details via DM.</t>
         </is>
       </c>
     </row>
@@ -37214,7 +37189,7 @@
       </c>
       <c r="O582" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com sent a polite private message to a user, asking them to review a private message sent earlier.</t>
         </is>
       </c>
     </row>
@@ -37276,7 +37251,7 @@
       </c>
       <c r="O583" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs a partner that it cannot provide support from its Social Media Team and directs them to an alternative contact link.</t>
         </is>
       </c>
     </row>
@@ -37343,7 +37318,7 @@
       </c>
       <c r="O584" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs a customer that only the accommodation can issue invoices and offers to help contact the property.</t>
         </is>
       </c>
     </row>
@@ -37408,7 +37383,7 @@
       </c>
       <c r="O585" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint about delayed support, offering to collect reservation details via private message to resolve the issue.</t>
         </is>
       </c>
     </row>
@@ -37469,12 +37444,12 @@
       </c>
       <c r="N586" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O586" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com addresses a customer’s concern about an additional charge, requesting booking details via private message for review.</t>
         </is>
       </c>
     </row>
@@ -37522,22 +37497,22 @@
       </c>
       <c r="L587" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M587" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N587" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O587" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Sky Bird Travel is promoting a 25% commission on travel insurance for agents, positioning it as a value‑add that protects travelers and boosts revenue.</t>
         </is>
       </c>
     </row>
@@ -37593,22 +37568,22 @@
       </c>
       <c r="L588" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M588" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N588" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O588" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Sky Bird Travel is promoting a 25% commission opportunity on travel insurance through its WINGS platform, positioning it as a value‑add for travel agents to enhance itineraries and revenue.</t>
         </is>
       </c>
     </row>
@@ -37654,7 +37629,7 @@
       </c>
       <c r="L589" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M589" t="inlineStr">
@@ -37669,7 +37644,7 @@
       </c>
       <c r="O589" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Navan shares a playful tweet highlighting a new connection or hire, indicating active engagement with industry talent.</t>
         </is>
       </c>
     </row>
@@ -37732,12 +37707,12 @@
       </c>
       <c r="L590" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M590" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N590" t="inlineStr">
@@ -37747,7 +37722,7 @@
       </c>
       <c r="O590" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Navan promotes a 48‑hour San Francisco itinerary curated by Gary, SVP of Global Account Management at Adyen, showcasing travel recommendations and highlighting the service.</t>
         </is>
       </c>
     </row>
@@ -37810,22 +37785,22 @@
       </c>
       <c r="L591" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M591" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N591" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O591" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>TravelPerk unveiled Entry Ready, an AI-native feature that lets users check visa requirements, receive guidance, pay for eVisas, and complete applications directly within the platform, simplifying international travel for business travelers.</t>
         </is>
       </c>
     </row>
@@ -37956,7 +37931,7 @@
       </c>
       <c r="O593" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex sends a friendly message to @axrahman, possibly indicating a forthcoming meeting or collaboration.</t>
         </is>
       </c>
     </row>
@@ -38002,22 +37977,22 @@
       </c>
       <c r="L594" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M594" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N594" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O594" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex announces a partnership with Cursor, indicating a collaborative effort to enhance services.</t>
         </is>
       </c>
     </row>
@@ -38079,22 +38054,22 @@
       </c>
       <c r="L595" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M595" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N595" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O595" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Airbnb announces the addition of rental car bookings, expanding its travel services to include vehicle rentals directly through its platform.</t>
         </is>
       </c>
     </row>
@@ -38155,7 +38130,7 @@
       </c>
       <c r="O596" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a private message from user @zd1tx, inviting them to review the response.</t>
         </is>
       </c>
     </row>
@@ -38219,7 +38194,7 @@
       </c>
       <c r="O597" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user’s accident with empathetic support, requesting booking details to assist with insurance and reservation inquiries.</t>
         </is>
       </c>
     </row>
@@ -38284,7 +38259,7 @@
       </c>
       <c r="O598" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a delayed response to a complaint and requests booking details via DM to investigate the issue.</t>
         </is>
       </c>
     </row>
@@ -38345,7 +38320,7 @@
       </c>
       <c r="O599" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user, suggesting they send the required information via direct message for review.</t>
         </is>
       </c>
     </row>
@@ -38397,7 +38372,7 @@
       </c>
       <c r="L600" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M600" t="inlineStr">
@@ -38407,12 +38382,12 @@
       </c>
       <c r="N600" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O600" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is requesting private booking details from users, which appears to be a phishing attempt.</t>
         </is>
       </c>
     </row>
@@ -38472,12 +38447,12 @@
       </c>
       <c r="N601" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O601" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is addressing a user’s complaint about a compromised account and requesting personal details to investigate the incident.</t>
         </is>
       </c>
     </row>
@@ -38538,7 +38513,7 @@
       </c>
       <c r="O602" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs a customer that their case has been updated via email and invites them to review the information.</t>
         </is>
       </c>
     </row>
@@ -38599,7 +38574,7 @@
       </c>
       <c r="O603" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint about misinformation from a third party, clarifying that reservations can only be made via their website or app and advising against engaging with third parties.</t>
         </is>
       </c>
     </row>
@@ -38666,7 +38641,7 @@
       </c>
       <c r="O604" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs a customer that the decision to waive potential cancellation fees is solely at the property’s discretion and requests confirmation details to review the request.</t>
         </is>
       </c>
     </row>
@@ -38732,7 +38707,7 @@
       </c>
       <c r="O605" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint, offering to review the issue and providing contact details for immediate assistance.</t>
         </is>
       </c>
     </row>
@@ -38797,7 +38772,7 @@
       </c>
       <c r="O606" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is offering customers instructions on how to contact 24/7 support and send private messages with booking details for assistance.</t>
         </is>
       </c>
     </row>
@@ -38848,7 +38823,7 @@
       </c>
       <c r="L607" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M607" t="inlineStr">
@@ -38858,12 +38833,12 @@
       </c>
       <c r="N607" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="O607" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>The post appears to be a phishing attempt, requesting private booking details from users.</t>
         </is>
       </c>
     </row>
@@ -38924,7 +38899,7 @@
       </c>
       <c r="O608" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a direct message from user @pala77liverpool, indicating ongoing communication.</t>
         </is>
       </c>
     </row>
@@ -38985,7 +38960,7 @@
       </c>
       <c r="O609" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs a user that flight reservations cannot be handled via social media and directs them to contact the Flights team through a link or phone.</t>
         </is>
       </c>
     </row>
@@ -39050,7 +39025,7 @@
       </c>
       <c r="O610" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a late response and a cancelled booking, asking the customer to DM booking details for resolution.</t>
         </is>
       </c>
     </row>
@@ -39116,7 +39091,7 @@
       </c>
       <c r="O611" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a customer’s disappointment and requests private details to review the reservation.</t>
         </is>
       </c>
     </row>
@@ -39178,7 +39153,7 @@
       </c>
       <c r="O612" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs users that it cannot process car rental reservations through social media and directs them to a specialized team via a provided link.</t>
         </is>
       </c>
     </row>
@@ -39239,7 +39214,7 @@
       </c>
       <c r="O613" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a delayed response to a user on X, citing a high volume of social media inquiries.</t>
         </is>
       </c>
     </row>
@@ -39300,7 +39275,7 @@
       </c>
       <c r="O614" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s private message, thanking them and informing them that their inquiry has been addressed.</t>
         </is>
       </c>
     </row>
@@ -39366,7 +39341,7 @@
       </c>
       <c r="O615" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com explains its social media support workflow for accommodation bookings and directs users to other channels for flights, taxis, or insurance inquiries.</t>
         </is>
       </c>
     </row>
@@ -39414,22 +39389,22 @@
       </c>
       <c r="L616" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M616" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N616" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O616" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>TravelPerk introduces Perk Spend, a new feature that merges travel and spend data to keep surprise charges on the pitch rather than in expense reports.</t>
         </is>
       </c>
     </row>
@@ -39480,7 +39455,7 @@
       </c>
       <c r="M617" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Tech Updates</t>
         </is>
       </c>
       <c r="N617" t="inlineStr">
@@ -39490,7 +39465,7 @@
       </c>
       <c r="O617" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp shares a link to content from @KlausCodes, likely highlighting a new feature or collaboration.</t>
         </is>
       </c>
     </row>
@@ -39536,7 +39511,7 @@
       </c>
       <c r="L618" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M618" t="inlineStr">
@@ -39551,7 +39526,7 @@
       </c>
       <c r="O618" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex tweets a lighthearted remark about San Francisco’s summer, indicating a casual engagement with the local vibe.</t>
         </is>
       </c>
     </row>
@@ -39597,12 +39572,12 @@
       </c>
       <c r="L619" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M619" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N619" t="inlineStr">
@@ -39612,7 +39587,7 @@
       </c>
       <c r="O619" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex teases an upcoming product or initiative, expressing confidence and readiness.</t>
         </is>
       </c>
     </row>
@@ -39658,7 +39633,7 @@
       </c>
       <c r="L620" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M620" t="inlineStr">
@@ -39673,7 +39648,7 @@
       </c>
       <c r="O620" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Brex posts a playful congratulatory message to @linderps, calling it a 'Grammy' award.</t>
         </is>
       </c>
     </row>
@@ -39724,12 +39699,12 @@
       </c>
       <c r="L621" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M621" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N621" t="inlineStr">
@@ -39739,7 +39714,7 @@
       </c>
       <c r="O621" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Expedia promotes Slovenia as a hidden European mountain escape, highlighting scenic activities, local culture, and off-grid accommodations, encouraging bookings via a link.</t>
         </is>
       </c>
     </row>
@@ -39796,22 +39771,22 @@
       </c>
       <c r="L622" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M622" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N622" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O622" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Expedia Group announced a dynamic creative production system powered by Google AI tools that increased creative effectiveness by 800%, enabling the creation of 800 hyper‑personalized ad variations daily.</t>
         </is>
       </c>
     </row>
@@ -39872,7 +39847,7 @@
       </c>
       <c r="O623" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s message on X, indicating a routine customer support interaction.</t>
         </is>
       </c>
     </row>
@@ -39937,7 +39912,7 @@
       </c>
       <c r="O624" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a dissatisfied customer, explaining its refund policy and offering to discuss the complaint with the accommodation.</t>
         </is>
       </c>
     </row>
@@ -39998,7 +39973,7 @@
       </c>
       <c r="O625" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com clarifies that flight bookings cannot be processed through social media and directs users to contact the Flights team via a provided link or phone numbers.</t>
         </is>
       </c>
     </row>
@@ -40059,7 +40034,7 @@
       </c>
       <c r="O626" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer inquiry, directing them to contact via DM for case review.</t>
         </is>
       </c>
     </row>
@@ -40120,7 +40095,7 @@
       </c>
       <c r="O627" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is following up with a user who has not yet provided all booking details, requesting the missing information via direct message.</t>
         </is>
       </c>
     </row>
@@ -40171,7 +40146,7 @@
       </c>
       <c r="L628" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M628" t="inlineStr">
@@ -40186,7 +40161,7 @@
       </c>
       <c r="O628" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is responding to a customer inquiry about a car rental reservation, requesting personal details via private message to assist.</t>
         </is>
       </c>
     </row>
@@ -40247,7 +40222,7 @@
       </c>
       <c r="O629" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs users that flight assistance cannot be provided via X and directs them to the Flights team through a link or phone numbers.</t>
         </is>
       </c>
     </row>
@@ -40311,7 +40286,7 @@
       </c>
       <c r="O630" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com reminds customers to include the confirmation number, confidential code, and traveler name when responding to reservation-related emails.</t>
         </is>
       </c>
     </row>
@@ -40373,7 +40348,7 @@
       </c>
       <c r="O631" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com acknowledges a user’s report and requests additional details via private message to investigate further.</t>
         </is>
       </c>
     </row>
@@ -40424,17 +40399,17 @@
       </c>
       <c r="M632" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Tech Updates</t>
         </is>
       </c>
       <c r="N632" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O632" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com addresses a user’s report of a suspicious email, apologizes for any concern, and warns against clicking links or making payments.</t>
         </is>
       </c>
     </row>
@@ -40500,7 +40475,7 @@
       </c>
       <c r="O633" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer inquiry, offering support details and directing to their 24/7 customer service.</t>
         </is>
       </c>
     </row>
@@ -40565,7 +40540,7 @@
       </c>
       <c r="O634" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responded to a user’s complaint about an extra charge, offering to resolve the issue via direct message.</t>
         </is>
       </c>
     </row>
@@ -40633,7 +40608,7 @@
       </c>
       <c r="O635" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com clarifies cancellation procedures and fee policies for customers.</t>
         </is>
       </c>
     </row>
@@ -40694,7 +40669,7 @@
       </c>
       <c r="O636" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a direct message from user @hakhak20212021, indicating a private customer interaction.</t>
         </is>
       </c>
     </row>
@@ -40755,7 +40730,7 @@
       </c>
       <c r="O637" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint, offering alternative contact for flight assistance.</t>
         </is>
       </c>
     </row>
@@ -40820,7 +40795,7 @@
       </c>
       <c r="O638" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is responding to a user’s concern and requesting booking details via direct message for further review.</t>
         </is>
       </c>
     </row>
@@ -40881,7 +40856,7 @@
       </c>
       <c r="O639" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s direct message, indicating routine customer support engagement.</t>
         </is>
       </c>
     </row>
@@ -40932,7 +40907,7 @@
       </c>
       <c r="M640" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Partnership and Acquisitions</t>
         </is>
       </c>
       <c r="N640" t="inlineStr">
@@ -40942,7 +40917,7 @@
       </c>
       <c r="O640" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com contacted a potential partner, informing them of a private message with additional details about their file.</t>
         </is>
       </c>
     </row>
@@ -41004,7 +40979,7 @@
       </c>
       <c r="O641" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s direct message, indicating routine customer support engagement.</t>
         </is>
       </c>
     </row>
@@ -41076,7 +41051,7 @@
       </c>
       <c r="O642" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is offering customer support via private messages for reservation and account issues.</t>
         </is>
       </c>
     </row>
@@ -41126,7 +41101,7 @@
       </c>
       <c r="L643" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M643" t="inlineStr">
@@ -41141,7 +41116,7 @@
       </c>
       <c r="O643" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Sky Bird Travel promotes booking with a travel advisor for expert support, emphasizing peace of mind and personalized service to encourage confident travel.</t>
         </is>
       </c>
     </row>
@@ -41199,7 +41174,7 @@
       </c>
       <c r="L644" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M644" t="inlineStr">
@@ -41214,7 +41189,7 @@
       </c>
       <c r="O644" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Sky Bird Travel highlights the benefits of booking with a travel advisor, emphasizing peace of mind, personalized support, and up-to-date travel information for travelers.</t>
         </is>
       </c>
     </row>
@@ -41269,12 +41244,12 @@
       </c>
       <c r="L645" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M645" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N645" t="inlineStr">
@@ -41284,7 +41259,7 @@
       </c>
       <c r="O645" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Navan's LinkedIn post expresses frustration with the onboarding process, implying challenges in getting clients to onboard.</t>
         </is>
       </c>
     </row>
@@ -41345,7 +41320,7 @@
       </c>
       <c r="O646" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp posted a brief mention of Elon Musk without additional context or details.</t>
         </is>
       </c>
     </row>
@@ -41396,7 +41371,7 @@
       </c>
       <c r="M647" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Tech Updates</t>
         </is>
       </c>
       <c r="N647" t="inlineStr">
@@ -41406,7 +41381,7 @@
       </c>
       <c r="O647" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp posts a question about the authenticity of Grok, indicating curiosity or inquiry into a new technology or product.</t>
         </is>
       </c>
     </row>
@@ -41467,7 +41442,7 @@
       </c>
       <c r="O648" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp tweets a question to @rahulgs and @grok asking if a statement is true.</t>
         </is>
       </c>
     </row>
@@ -41547,12 +41522,12 @@
       </c>
       <c r="L649" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M649" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N649" t="inlineStr">
@@ -41562,7 +41537,7 @@
       </c>
       <c r="O649" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Airbnb humorously promotes a Paris apartment listing, encouraging bookings with playful language and a light‑hearted marketing tone.</t>
         </is>
       </c>
     </row>
@@ -41612,12 +41587,12 @@
       </c>
       <c r="L650" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M650" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N650" t="inlineStr">
@@ -41627,7 +41602,7 @@
       </c>
       <c r="O650" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Expedia is promoting a new travel package to Norway, highlighting fjords, islands, and unique cabin stays, encouraging bookings via a dedicated link.</t>
         </is>
       </c>
     </row>
@@ -41693,7 +41668,7 @@
       </c>
       <c r="O651" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com addresses a customer’s issue with a missing booking confirmation, offering investigation and potential refund while explaining possible causes.</t>
         </is>
       </c>
     </row>
@@ -41754,7 +41729,7 @@
       </c>
       <c r="O652" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer’s issue via direct message, offering assistance and directing them to 24/7 phone support.</t>
         </is>
       </c>
     </row>
@@ -41815,12 +41790,12 @@
       </c>
       <c r="N653" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O653" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer’s complaint about a delayed refund, apologizes for the inconvenience, and requests booking details via DM to investigate the issue.</t>
         </is>
       </c>
     </row>
@@ -41881,7 +41856,7 @@
       </c>
       <c r="O654" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a direct message from user @SudharshananJa1.</t>
         </is>
       </c>
     </row>
@@ -41942,7 +41917,7 @@
       </c>
       <c r="O655" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replies to a user on X, apologizing for a delayed response due to high volume of cases.</t>
         </is>
       </c>
     </row>
@@ -42009,7 +41984,7 @@
       </c>
       <c r="O656" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a delayed response and guides the customer on how to verify accommodation status and contact options.</t>
         </is>
       </c>
     </row>
@@ -42058,7 +42033,7 @@
       </c>
       <c r="L657" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M657" t="inlineStr">
@@ -42073,7 +42048,7 @@
       </c>
       <c r="O657" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s complaint about a negative experience, offering to resolve the issue via direct message and requesting additional booking details.</t>
         </is>
       </c>
     </row>
@@ -42134,7 +42109,7 @@
       </c>
       <c r="O658" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responded to a user query by providing its India customer care phone number.</t>
         </is>
       </c>
     </row>
@@ -42201,7 +42176,7 @@
       </c>
       <c r="O659" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is responding to a customer inquiry about a car rental reservation, requesting booking details via private message.</t>
         </is>
       </c>
     </row>
@@ -42262,7 +42237,7 @@
       </c>
       <c r="O660" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a private message from a user, offering follow-up assistance.</t>
         </is>
       </c>
     </row>
@@ -42312,7 +42287,7 @@
       </c>
       <c r="L661" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M661" t="inlineStr">
@@ -42327,7 +42302,7 @@
       </c>
       <c r="O661" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer query, offering assistance and requesting reservation details via DM.</t>
         </is>
       </c>
     </row>
@@ -42388,7 +42363,7 @@
       </c>
       <c r="O662" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a dissatisfied user, offering to resolve the issue via direct message.</t>
         </is>
       </c>
     </row>
@@ -42454,7 +42429,7 @@
       </c>
       <c r="O663" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com explains that cancellation fees are set by accommodations and directs customers to private messaging or phone support for assistance.</t>
         </is>
       </c>
     </row>
@@ -42505,7 +42480,7 @@
       </c>
       <c r="L664" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M664" t="inlineStr">
@@ -42520,7 +42495,7 @@
       </c>
       <c r="O664" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com addresses a customer complaint about a poor stay, apologizes, and directs the customer to an email response while offering further assistance via direct message.</t>
         </is>
       </c>
     </row>
@@ -42581,7 +42556,7 @@
       </c>
       <c r="O665" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user’s inquiry by warning against sharing reservation PIN codes publicly and encourages the user to delete the comment and contact them privately for assistance.</t>
         </is>
       </c>
     </row>
@@ -42643,7 +42618,7 @@
       </c>
       <c r="O666" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is requesting a PIN code and full guest name from a customer to verify a booking for security purposes.</t>
         </is>
       </c>
     </row>
@@ -42707,7 +42682,7 @@
       </c>
       <c r="O667" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer inquiry, offering to resend the final outcome upon request.</t>
         </is>
       </c>
     </row>
@@ -42768,7 +42743,7 @@
       </c>
       <c r="O668" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s direct message offering further support.</t>
         </is>
       </c>
     </row>
@@ -42834,7 +42809,7 @@
       </c>
       <c r="O669" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com addresses a user’s complaint about potential misinformation on a listed property, offering to investigate and remove the property if necessary.</t>
         </is>
       </c>
     </row>
@@ -42895,7 +42870,7 @@
       </c>
       <c r="O670" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint on X, offering assistance and directing the user to their 24/7 support line.</t>
         </is>
       </c>
     </row>
@@ -42941,7 +42916,7 @@
       </c>
       <c r="L671" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M671" t="inlineStr">
@@ -42956,7 +42931,7 @@
       </c>
       <c r="O671" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Ramp's tweet hints at a compliance issue, labeling it as 'Crime but compliant', suggesting potential regulatory concerns.</t>
         </is>
       </c>
     </row>
@@ -43017,7 +42992,7 @@
       </c>
       <c r="O672" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com sent a private message to user @cactushoney12, requesting them to check it.</t>
         </is>
       </c>
     </row>
@@ -43067,7 +43042,7 @@
       </c>
       <c r="L673" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M673" t="inlineStr">
@@ -43077,12 +43052,12 @@
       </c>
       <c r="N673" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O673" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a customer’s frustration and explains that their team cannot see reservation details without direct information, requesting the customer to provide details for further assistance.</t>
         </is>
       </c>
     </row>
@@ -43143,7 +43118,7 @@
       </c>
       <c r="O674" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s direct message, indicating routine customer support activity.</t>
         </is>
       </c>
     </row>
@@ -43208,7 +43183,7 @@
       </c>
       <c r="O675" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is offering customer support for outstanding refunds, requesting booking details via direct message.</t>
         </is>
       </c>
     </row>
@@ -43272,7 +43247,7 @@
       </c>
       <c r="O676" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer on X, requesting personal details to investigate a complaint.</t>
         </is>
       </c>
     </row>
@@ -43333,7 +43308,7 @@
       </c>
       <c r="O677" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user’s inquiry about an Agoda reservation, directing them to contact Agoda directly for assistance.</t>
         </is>
       </c>
     </row>
@@ -43403,7 +43378,7 @@
       </c>
       <c r="O678" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint, explaining that cancellation and refund policies are set by the accommodation and requesting booking details for further investigation.</t>
         </is>
       </c>
     </row>
@@ -43467,7 +43442,7 @@
       </c>
       <c r="O679" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com addresses a customer complaint about a reservation in Columbus, Ohio, apologizing for the inconvenience and offering to collect details via DM while directing the user to 24/7 support.</t>
         </is>
       </c>
     </row>
@@ -43528,7 +43503,7 @@
       </c>
       <c r="O680" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com sent a private message to user @MuathMuhammad, asking them to check the message.</t>
         </is>
       </c>
     </row>
@@ -43589,7 +43564,7 @@
       </c>
       <c r="O681" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user on X, acknowledging their concern and directing them to check their direct message for further assistance.</t>
         </is>
       </c>
     </row>
@@ -43650,7 +43625,7 @@
       </c>
       <c r="O682" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied to a user’s inquiry via direct message, directing them to check their messages for additional support.</t>
         </is>
       </c>
     </row>
@@ -43717,7 +43692,7 @@
       </c>
       <c r="O683" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer’s car rental damage claim, requesting booking details via private message.</t>
         </is>
       </c>
     </row>
@@ -43778,7 +43753,7 @@
       </c>
       <c r="O684" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replied privately to a user on X, notifying them that a response has been sent.</t>
         </is>
       </c>
     </row>
@@ -43834,12 +43809,12 @@
       </c>
       <c r="N685" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O685" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes to a customer for a frustrating support experience and invites them to discuss the issue privately.</t>
         </is>
       </c>
     </row>
@@ -43903,7 +43878,7 @@
       </c>
       <c r="O686" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is following up with a customer about a pending refund, requesting confirmation details via direct message.</t>
         </is>
       </c>
     </row>
@@ -43954,17 +43929,17 @@
       </c>
       <c r="M687" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Tech Updates</t>
         </is>
       </c>
       <c r="N687" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O687" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com advises a user to avoid sharing reservation PIN codes publicly and to delete the comment, urging a private discussion for security.</t>
         </is>
       </c>
     </row>
@@ -44025,7 +44000,7 @@
       </c>
       <c r="O688" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com sent a private message to user Karina Parvanova, likely for a follow-up or support.</t>
         </is>
       </c>
     </row>
@@ -44086,7 +44061,7 @@
       </c>
       <c r="O689" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com sent a direct message to user @Patreus7575, requesting them to check their DM.</t>
         </is>
       </c>
     </row>
@@ -44137,7 +44112,7 @@
       </c>
       <c r="L690" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M690" t="inlineStr">
@@ -44147,12 +44122,12 @@
       </c>
       <c r="N690" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O690" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com clarifies that property availability is controlled by the properties themselves and offers support for customers encountering fraudulent listings.</t>
         </is>
       </c>
     </row>
@@ -44213,7 +44188,7 @@
       </c>
       <c r="O691" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com sent a private message to user @KatarinaHill2, likely for outreach or support purposes.</t>
         </is>
       </c>
     </row>
@@ -44626,7 +44601,7 @@
       </c>
       <c r="O697" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a flight cancellation and refund delay, explains the inability to assist via social media, and directs the customer to the flight support team.</t>
         </is>
       </c>
     </row>
@@ -44691,7 +44666,7 @@
       </c>
       <c r="O698" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com replies to a user’s inquiry, asking for a confidential code and traveler name to review the case.</t>
         </is>
       </c>
     </row>
@@ -44744,7 +44719,7 @@
       </c>
       <c r="L699" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M699" t="inlineStr">
@@ -44759,7 +44734,7 @@
       </c>
       <c r="O699" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologizes for a delayed response to a customer complaint and provides instructions for private messaging and contact details.</t>
         </is>
       </c>
     </row>
@@ -44806,7 +44781,7 @@
       </c>
       <c r="L700" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M700" t="inlineStr">
@@ -44821,7 +44796,7 @@
       </c>
       <c r="O700" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com apologized to a user for a flight cancellation and delayed response, indicating the issue was handled via a private message.</t>
         </is>
       </c>
     </row>
@@ -44883,7 +44858,7 @@
       </c>
       <c r="O701" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com publicly acknowledges a user’s private message, expressing empathy about an incident.</t>
         </is>
       </c>
     </row>
@@ -44948,7 +44923,7 @@
       </c>
       <c r="O702" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a user’s complaint about a booking issue, offering a refund and requesting confirmation details via private message.</t>
         </is>
       </c>
     </row>
@@ -44994,7 +44969,7 @@
       </c>
       <c r="L703" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M703" t="inlineStr">
@@ -45004,12 +44979,12 @@
       </c>
       <c r="N703" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="O703" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com informs users that they cannot help with verification issues and directs them to a link for listing properties.</t>
         </is>
       </c>
     </row>
@@ -45070,7 +45045,7 @@
       </c>
       <c r="O704" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com sent a direct message to user @MiriamFeldman12, inviting them to review the reply for more details.</t>
         </is>
       </c>
     </row>
@@ -45131,7 +45106,7 @@
       </c>
       <c r="O705" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com sent a private message to user @medactif, likely for support or communication.</t>
         </is>
       </c>
     </row>
@@ -45181,7 +45156,7 @@
       </c>
       <c r="L706" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="M706" t="inlineStr">
@@ -45196,7 +45171,7 @@
       </c>
       <c r="O706" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint about a pending refund, offering to investigate via DM and directing the customer to 24/7 support.</t>
         </is>
       </c>
     </row>
@@ -45260,7 +45235,7 @@
       </c>
       <c r="O707" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer’s difficulty reaching support, offering to investigate the booking and requesting confirmation details.</t>
         </is>
       </c>
     </row>
@@ -45326,7 +45301,7 @@
       </c>
       <c r="O708" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com responds to a customer complaint about a reservation not honored, clarifying that property owners control availability and offering steps for resolution.</t>
         </is>
       </c>
     </row>
@@ -45387,7 +45362,7 @@
       </c>
       <c r="O709" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com acknowledges a customer’s negative experience and directs them to a private message for resolution.</t>
         </is>
       </c>
     </row>
@@ -45450,7 +45425,7 @@
       </c>
       <c r="O710" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com clarifies its language support on X, offering assistance in several languages but not Arabic, and directs Arabic-speaking users to a local contact number.</t>
         </is>
       </c>
     </row>
@@ -45511,7 +45486,7 @@
       </c>
       <c r="O711" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com acknowledges a customer’s delayed response issue and requests a private message for further assistance.</t>
         </is>
       </c>
     </row>
@@ -45572,7 +45547,7 @@
       </c>
       <c r="O712" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com sent a private message to user @cactushoney12, prompting them to check their private message.</t>
         </is>
       </c>
     </row>
@@ -45633,7 +45608,7 @@
       </c>
       <c r="O713" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com is following up with a user to request additional details for next steps.</t>
         </is>
       </c>
     </row>
@@ -45700,7 +45675,7 @@
       </c>
       <c r="O714" t="inlineStr">
         <is>
-          <t>Failed to analyze post via LLM.</t>
+          <t>Booking.com for Travel Agents outlines its social media support process for accommodation bookings, providing required details for DMs and directing users to phone support for urgent needs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
style: implement dynamic social signals filters and fix failed LLM post insights
</commit_message>
<xml_diff>
--- a/News_Dashboard/data/social_media_posts.xlsx
+++ b/News_Dashboard/data/social_media_posts.xlsx
@@ -4137,7 +4137,10 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>[Transcript unavailable: 
+Could not retrieve a transcript for the video https://www.youtube.com/watch?v=achyqRan3xI! This is most likely caused by:
+Subtitles are disabled for this video
+If you are sure that the described cause is not responsible for this error and that a transcript should be retrievable, please create an issue at https://github.com/jdepoix/youtube-transcript-api/issues. Please add which version of youtube_transcript_api you are using and provide the information needed to replicate the error. Also make sure that there are no open issues which already describe your problem!]</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -4147,22 +4150,22 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>Transcript not available.</t>
         </is>
       </c>
     </row>
@@ -4347,7 +4350,10 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>[Transcript unavailable: 
+Could not retrieve a transcript for the video https://www.youtube.com/watch?v=HKOtGZP1Utc! This is most likely caused by:
+Subtitles are disabled for this video
+If you are sure that the described cause is not responsible for this error and that a transcript should be retrievable, please create an issue at https://github.com/jdepoix/youtube-transcript-api/issues. Please add which version of youtube_transcript_api you are using and provide the information needed to replicate the error. Also make sure that there are no open issues which already describe your problem!]</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -7374,7 +7380,10 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>[Transcript unavailable: 
+Could not retrieve a transcript for the video https://www.youtube.com/watch?v=PAkOQITfIiA! This is most likely caused by:
+Subtitles are disabled for this video
+If you are sure that the described cause is not responsible for this error and that a transcript should be retrievable, please create an issue at https://github.com/jdepoix/youtube-transcript-api/issues. Please add which version of youtube_transcript_api you are using and provide the information needed to replicate the error. Also make sure that there are no open issues which already describe your problem!]</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7384,22 +7393,22 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>Transcript not available for the requested video.</t>
         </is>
       </c>
     </row>
@@ -9267,7 +9276,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>[music] &gt;&gt; Oh. Hey, what's up?</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -9277,12 +9286,12 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N140" t="inlineStr">
@@ -9290,7 +9299,11 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="O140" t="inlineStr"/>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>Brex showcases a new feature that dramatically speeds up the month‑end close process, reducing the time from 14 days to just minutes. The video highlights how this improvement streamlines finance operations and boosts productivity for users.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -15273,7 +15286,10 @@
       </c>
       <c r="J232" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>Wait till you see this! With Expedia, The more you book, the more
+rewards you can unlock. and the more rewards you
+unlock, the more you get to
+enjoy whatever this is.</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -15283,12 +15299,12 @@
       </c>
       <c r="L232" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M232" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N232" t="inlineStr">
@@ -15298,7 +15314,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>The video promotes Expedia’s rewards program, highlighting that the more customers book, the more rewards they unlock, enhancing their travel experience.</t>
         </is>
       </c>
     </row>
@@ -35084,7 +35100,7 @@
       </c>
       <c r="J550" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>Things have improved my life from a user's perspective and a finance perspective. Obviously, compliance, a lot of control, so my accounting team's happy, my controllers are happy, my CFO's happy, but the business is happy. The business feels like their data is clean now. &gt;&gt; [music] &gt;&gt; Um the users are being listened to. We've automated a lot of um manual steps uh through different tools um like the request tool to get pre-approvals. The excitement's growing. [music] They are now feeling like they can actually serve themselves. &gt;&gt; [music]</t>
         </is>
       </c>
       <c r="K550" t="inlineStr">
@@ -35094,12 +35110,12 @@
       </c>
       <c r="L550" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M550" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N550" t="inlineStr">
@@ -35109,7 +35125,7 @@
       </c>
       <c r="O550" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>The video highlights how Concur Expense has improved user and finance experiences by enhancing compliance, control, and data cleanliness. It showcases automation of manual steps, such as pre-approval requests, and emphasizes that users feel empowered to serve themselves, indicating growing excitement around the product.</t>
         </is>
       </c>
     </row>
@@ -35154,7 +35170,7 @@
       </c>
       <c r="J551" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>Concur Travel makes travel so much easier for our employees because they're it's it's it's a one-stop shop. It's not only saving me time, it's saving me approvers time because they're not having to then go review everything again. Prior to my joining the company, we were 25 to 30% over budget every [music] year in travel. Being able to see that data on a monthly basis and make shifts, we were actually on budget for the first time. &gt;&gt; [music]</t>
         </is>
       </c>
       <c r="K551" t="inlineStr">
@@ -35164,12 +35180,12 @@
       </c>
       <c r="L551" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M551" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N551" t="inlineStr">
@@ -35179,7 +35195,7 @@
       </c>
       <c r="O551" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>The video showcases a testimonial from a user of Concur Travel, highlighting how the platform simplifies travel management for employees and approvers, provides real‑time visibility into travel spend, and helped the company move from being 25‑30% over budget to staying on budget for the first time.</t>
         </is>
       </c>
     </row>
@@ -35224,7 +35240,7 @@
       </c>
       <c r="J552" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>sobre todo si automatiza procesos vida de todos pero debe funcionar que ya tienes cuando los datos sin trabas entre sistemas tus procesos se integran y tu empresa opera como debe por eso SAP Concur ofrece cientos de integraciones y conectores preconfigurados &gt;&gt; [music] &gt;&gt; al conectar nuestras soluciones con las tuyas tu empresa puede reducir costos su rentabilidad obtén visibilidad de datos de gasto actualizados [music] mejora el cumplimiento de políticas y elimina errores de procesos manuales lo mejor funcionan con cualquier ERP y si no ves una integración en nuestro [music] App Center no hay problema podemos crearla a la medida o tus desarrolladores pueden usar nuestras &gt;&gt; [music] &gt;&gt; abiertas para crear la que necesitas visita nuestra página de integraciones y aprovecha al máximo tu inversión en SAP Concur [music]</t>
         </is>
       </c>
       <c r="K552" t="inlineStr">
@@ -35234,12 +35250,12 @@
       </c>
       <c r="L552" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M552" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N552" t="inlineStr">
@@ -35249,7 +35265,7 @@
       </c>
       <c r="O552" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>El video presenta una guía para principiantes sobre las integraciones de SAP Concur, destacando cómo automatizan procesos, reducen costos, mejoran la visibilidad de datos de gasto, cumplen con políticas y eliminan errores manuales. Se menciona la disponibilidad de cientos de integraciones preconfiguradas, la posibilidad de crear integraciones personalizadas y el uso de conectores abiertos para desarrolladores.</t>
         </is>
       </c>
     </row>
@@ -35294,7 +35310,7 @@
       </c>
       <c r="J553" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>Concur Invoice really is such an important component of what I do in my [music] everyday job. It allows customization of workflows. It allows us to monitor our processes through various like the invoice manager dashboard, things of that nature. And it really does enable us to push invoices out faster, to get those payment cycle times down as low as possible, and also [music] not burden our approvers and our reviewers with just tedious work. &gt;&gt; [music] &gt;&gt; It allows them to make actionable decisions instead of just cranking through a list of things that they [music] have to get done today.</t>
         </is>
       </c>
       <c r="K553" t="inlineStr">
@@ -35304,12 +35320,12 @@
       </c>
       <c r="L553" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M553" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Product Announcement</t>
         </is>
       </c>
       <c r="N553" t="inlineStr">
@@ -35319,7 +35335,7 @@
       </c>
       <c r="O553" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>The video showcases Concur Invoice as a key tool in the speaker’s daily work, highlighting its ability to customize workflows, monitor processes via an invoice manager dashboard, accelerate invoice processing, shorten payment cycle times, and reduce the administrative burden on approvers and reviewers.</t>
         </is>
       </c>
     </row>
@@ -35364,7 +35380,7 @@
       </c>
       <c r="J554" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>[music] &gt;&gt; Prior to my joining the company, we were 25% over budget every year in travel. After we started pulling the data, and of course there were some other factors that went into [music] to cost saving as well, but being able to see that data on a monthly basis and make shifts, &gt;&gt; [music] &gt;&gt; we were actually on budget for the first time in 2024 and 2025. Being able to pull reporting from Concur and present it to the management team, it was the first [music] time that they had seen data at that granular level as opposed to just a bottom line budget impact. [music] So, it was extremely impactful. &gt;&gt; [music] &gt;&gt; We could [music] look at where our compliance issues were. So, where we were seeing some unnecessary spend, we could tweak the [music] policy to say, "Hey, you know, maybe we need to limit that spend or remove it altogether." &gt;&gt; [music]</t>
         </is>
       </c>
       <c r="K554" t="inlineStr">
@@ -35374,12 +35390,12 @@
       </c>
       <c r="L554" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M554" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Tech Updates</t>
         </is>
       </c>
       <c r="N554" t="inlineStr">
@@ -35389,7 +35405,7 @@
       </c>
       <c r="O554" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>The video discusses how Meteor Education leveraged data visibility, verification, and AI tools—particularly Concur reporting—to transform its travel spend management. By monitoring monthly data, identifying compliance issues, and adjusting policies, the company moved from being 25% over budget to staying on budget for the first time in 2024 and 2025, highlighting significant cost savings and operational impact.</t>
         </is>
       </c>
     </row>
@@ -37845,7 +37861,7 @@
       </c>
       <c r="J592" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>[music] &gt;&gt; With the intelligence [music] reporting tool within Concur, &gt;&gt; [music] &gt;&gt; we can get in there. We get a lot of visibility into what [music] our spend is. We got reports for spend by category, spend by person, spend by department. [music] We've created a bunch of custom reports, which I think is great. And then we have of course the standard [music] reports for helping us with the accruals on the finance side and the month and the year credit card reconciliation. &gt;&gt; [music] &gt;&gt; That's a lot easier just running the report. Seeing what was submitted, what wasn't submitted. [music] And then wasn't submitted and the month you accrued, then you follow up with the people and get them to finish everything and then the reconciliation [music] of the statements is done. That's been very clean since we implemented it. We're very happy with that. &gt;&gt; [music] &gt;&gt; One advantage we do have again what I see from Concur side is [music] that we can have reporting extracts. So reporting intelligence actually is one of the very powerful Cognos database that we currently use and [music] I think it's a fantastic data repository where pretty much you get if you have the right reporting and the right &gt;&gt; [music] &gt;&gt; way or the right requirements written down, I think we get a very good &gt;&gt; [music] &gt;&gt; report out of it. We get Today currently for us we do get data extracted to our Power BI data warehouse &gt;&gt; [music] &gt;&gt; and we do generate some cool reports out of that. Today our finance teams, our spend [music] teams, AP teams and the leadership, they do view those data reports and they do view those [music] KPIs actually. From our Power BI reporting, but the underlying data everything is actually [music] coming out of Concur. &gt;&gt; When I started with Medair about 2 and 1/2 years ago, there was [music] no reporting being done. And that's one of the main reasons I was hired. So, being able to pull reporting from Concur and present it to the management team, it was the first [music] time that they had seen data at that granular level as opposed to just a bottom line budget impact. So, it was extremely impactful. We [music] could look at at at where our compliance issues were. We could look again at um [music] any policy changes we need to make based on that data. But, the biggest impact, um and I'm very proud of this, [music] is prior to my joining the company, we were 25 to 30% over budget every year in travel. After [music] we started pulling the data, and of course there were some other factors that went into to cost saving [music] as well, but being able to see that data on a monthly basis and make shifts, we were actually on budget for the first time. &gt;&gt; [music]</t>
         </is>
       </c>
       <c r="K592" t="inlineStr">
@@ -37855,12 +37871,12 @@
       </c>
       <c r="L592" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M592" t="inlineStr">
         <is>
-          <t>General Industry News</t>
+          <t>Tech Updates</t>
         </is>
       </c>
       <c r="N592" t="inlineStr">
@@ -37870,7 +37886,7 @@
       </c>
       <c r="O592" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>The video showcases how SAP Concur’s reporting and data extraction capabilities transformed travel spend management for a client. It highlights the ease of generating custom and standard reports, integrating Concur data with Power BI, and the resulting visibility that helped the organization reduce travel spend from 25‑30% over budget to on‑budget status. The speaker emphasizes the positive impact on compliance, policy adjustments, and overall financial oversight.</t>
         </is>
       </c>
     </row>
@@ -44233,7 +44249,7 @@
       </c>
       <c r="J692" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>Come on, come on. &gt;&gt; To make around $2,000 in a week, this man could walk 34 Chihuahuas every day. Or he could try putting his place on Airbnb.</t>
         </is>
       </c>
       <c r="K692" t="inlineStr">
@@ -44258,7 +44274,7 @@
       </c>
       <c r="O692" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>The video humorously compares the potential earnings of walking 34 Chihuahuas daily to listing a property on Airbnb, highlighting the financial prospects of each option.</t>
         </is>
       </c>
     </row>
@@ -44303,7 +44319,7 @@
       </c>
       <c r="J693" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>To make around $2,000 in a week, this couple could sell 2,000 lemonades. Oops. Or they could try putting their place on Airbnb.</t>
         </is>
       </c>
       <c r="K693" t="inlineStr">
@@ -44328,7 +44344,7 @@
       </c>
       <c r="O693" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>The video compares the potential earnings of a couple selling 2,000 lemonades in a week to listing their property on Airbnb, highlighting the financial opportunities of the Airbnb platform.</t>
         </is>
       </c>
     </row>
@@ -44373,7 +44389,7 @@
       </c>
       <c r="J694" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>To make around $2,000 in a week, this man could ref 56 soccer games. &gt;&gt; [cheering] &gt;&gt; Or, he could try putting his place on Airbnb. &gt;&gt; [cheering]</t>
         </is>
       </c>
       <c r="K694" t="inlineStr">
@@ -44398,7 +44414,7 @@
       </c>
       <c r="O694" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>The video humorously compares the potential earnings of refereeing 56 soccer games to listing a property on Airbnb, suggesting that the latter could be a more lucrative option for making around $2,000 in a week.</t>
         </is>
       </c>
     </row>
@@ -44443,7 +44459,7 @@
       </c>
       <c r="J695" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>This couple could make extra money this weekend by cat sitting for a whole lot of cats. &gt;&gt; [screaming] &gt;&gt; Or they could try putting their place on Airbnb.</t>
         </is>
       </c>
       <c r="K695" t="inlineStr">
@@ -44453,7 +44469,7 @@
       </c>
       <c r="L695" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="M695" t="inlineStr">
@@ -44468,7 +44484,7 @@
       </c>
       <c r="O695" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>The video humorously presents a couple weighing the option of earning extra money by cat‑sitting a large number of cats versus listing their home on Airbnb.</t>
         </is>
       </c>
     </row>
@@ -44513,7 +44529,7 @@
       </c>
       <c r="J696" t="inlineStr">
         <is>
-          <t>[Failed to fetch]</t>
+          <t>To make around $2,000 in a week, this woman could give 31 violin lessons. Or she could try putting her place on Airbnb.</t>
         </is>
       </c>
       <c r="K696" t="inlineStr">
@@ -44538,7 +44554,7 @@
       </c>
       <c r="O696" t="inlineStr">
         <is>
-          <t>Failed to analyze video transcript via LLM.</t>
+          <t>The video follows a woman who can earn about $2,000 in a week by either giving 31 violin lessons or listing her property on Airbnb, highlighting the choice between a traditional skill-based gig and a platform-based rental opportunity.</t>
         </is>
       </c>
     </row>

</xml_diff>